<commit_message>
refactor: use scenario no as data key
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -33,11 +33,6 @@
           <t>SCENARIOS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>DATA_ROW</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -58,9 +53,6 @@
           <t>Create booking room A</t>
         </is>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -68,21 +60,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cancel Booking</t>
+          <t>Create New Booking</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cancel booking</t>
+          <t>Create booking room B</t>
         </is>
-      </c>
-      <c r="E3">
-        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -91,21 +80,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Create New Booking</t>
+          <t>Cancel Booking</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Create booking room B</t>
+          <t>Cancel booking</t>
         </is>
-      </c>
-      <c r="E4">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: align scenario template headers
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -104,27 +104,37 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>STEP_NO</t>
+          <t>Testcase</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>KEYWORD</t>
+          <t>Run</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>OBJECT</t>
+          <t>Function</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>Object</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>DESCRIPTION</t>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -138,27 +148,37 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>STEP_NO</t>
+          <t>Testcase</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>KEYWORD</t>
+          <t>Run</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>OBJECT</t>
+          <t>Function</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>VALUE</t>
+          <t>Object</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>DESCRIPTION</t>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add scenario sheet parser
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -138,6 +138,228 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Login BRS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Login to BRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>txtUsername</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LOGIN_DATA[USERNAME]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Input username</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>txtPassword</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LOGIN_DATA[PASSWORD]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Input password</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>btnLogin</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Click login</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>verifyDisplayed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>lblDashboard</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Verify dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Create Booking</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Create booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>menuBooking</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Open booking menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>txtBookingTitle</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BOOKING_DATA[BOOKING_TITLE]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Input title</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>btnRoomByName</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BOOKING_DATA[ROOM_NAME]</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Select room</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>btnSubmitBooking</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Submit</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>verifyText</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>lblSuccessMessage</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Verify success</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -182,6 +404,172 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Login BRS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Login to BRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>txtUsername</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LOGIN_DATA[USERNAME]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Input username</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>txtPassword</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LOGIN_DATA[PASSWORD]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Input password</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>btnLogin</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Click login</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cancel Booking</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Cancel booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>menuBooking</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Open booking menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>btnCancelBooking</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BOOKING_DATA[BOOKING_ID]</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Cancel booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>verifyText</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>lblSuccessMessage</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Verify success</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
style: autofit excel template columns
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -1,6 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet name="SCENARIOS" sheetId="1" r:id="rId1"/>
     <sheet name="Create New Booking" sheetId="2" r:id="rId2"/>
@@ -9,86 +12,135 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <sz val="11.0"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="darkGray"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D4"/>
+  <cols>
+    <col min="1" max="1" width="10.0" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="19.265625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="21.49609375" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>RUN</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>ACTION</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>SCENARIOS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Create New Booking</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr" s="0">
         <is>
           <t>Create booking room A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="inlineStr" s="0">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr" s="0">
         <is>
           <t>Create New Booking</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr" s="0">
         <is>
           <t>Create booking room B</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" t="inlineStr" s="0">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr" s="0">
         <is>
           <t>Cancel Booking</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr" s="0">
         <is>
           <t>Cancel booking</t>
         </is>
@@ -100,261 +152,271 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G12"/>
+  <cols>
+    <col min="1" max="1" width="15.15625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="15.22265625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="18.078125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="34.265625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="12.01953125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="19.24609375" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Testcase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Login BRS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr" s="0">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr" s="0">
         <is>
           <t>Login to BRS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr" s="0">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr" s="0">
         <is>
           <t>txtUsername</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr" s="0">
         <is>
           <t>LOGIN_DATA[USERNAME]</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr" s="0">
         <is>
           <t>Input username</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr" s="0">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr" s="0">
         <is>
           <t>txtPassword</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="inlineStr" s="0">
         <is>
           <t>LOGIN_DATA[PASSWORD]</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr" s="0">
         <is>
           <t>Input password</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr" s="0">
         <is>
           <t>btnLogin</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr" s="0">
         <is>
           <t>Click login</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="inlineStr" s="0">
         <is>
           <t>verifyDisplayed</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="inlineStr" s="0">
         <is>
           <t>lblDashboard</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr" s="0">
         <is>
           <t>Verify dashboard</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="inlineStr" s="0">
         <is>
           <t>Create Booking</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="inlineStr" s="0">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" t="inlineStr" s="0">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="inlineStr" s="0">
         <is>
           <t>Create booking</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr" s="0">
         <is>
           <t>menuBooking</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="inlineStr" s="0">
         <is>
           <t>Open booking menu</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="inlineStr" s="0">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="inlineStr" s="0">
         <is>
           <t>txtBookingTitle</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" t="inlineStr" s="0">
         <is>
           <t>BOOKING_DATA[BOOKING_TITLE]</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="inlineStr" s="0">
         <is>
           <t>Input title</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr" s="0">
         <is>
           <t>btnRoomByName</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" t="inlineStr" s="0">
         <is>
           <t>BOOKING_DATA[ROOM_NAME]</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="inlineStr" s="0">
         <is>
           <t>Select room</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="inlineStr">
+      <c r="C11" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="inlineStr" s="0">
         <is>
           <t>btnSubmitBooking</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="inlineStr" s="0">
         <is>
           <t>Submit</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="inlineStr">
+      <c r="C12" t="inlineStr" s="0">
         <is>
           <t>verifyText</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="inlineStr" s="0">
         <is>
           <t>lblSuccessMessage</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" t="inlineStr" s="0">
         <is>
           <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="inlineStr" s="0">
         <is>
           <t>Verify success</t>
         </is>
@@ -366,205 +428,215 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G9"/>
+  <cols>
+    <col min="1" max="1" width="15.1484375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.8984375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="18.078125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="34.265625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="12.01953125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="19.24609375" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Testcase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Login BRS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr" s="0">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr" s="0">
         <is>
           <t>Login to BRS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr" s="0">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr" s="0">
         <is>
           <t>txtUsername</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr" s="0">
         <is>
           <t>LOGIN_DATA[USERNAME]</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr" s="0">
         <is>
           <t>Input username</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr" s="0">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr" s="0">
         <is>
           <t>txtPassword</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="inlineStr" s="0">
         <is>
           <t>LOGIN_DATA[PASSWORD]</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr" s="0">
         <is>
           <t>Input password</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr" s="0">
         <is>
           <t>btnLogin</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr" s="0">
         <is>
           <t>Click login</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="inlineStr" s="0">
         <is>
           <t>Cancel Booking</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="inlineStr" s="0">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" t="inlineStr" s="0">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr" s="0">
         <is>
           <t>Cancel booking</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr" s="0">
         <is>
           <t>menuBooking</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="inlineStr" s="0">
         <is>
           <t>Open booking menu</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="inlineStr" s="0">
         <is>
           <t>click</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr" s="0">
         <is>
           <t>btnCancelBooking</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" t="inlineStr" s="0">
         <is>
           <t>BOOKING_DATA[BOOKING_ID]</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="inlineStr" s="0">
         <is>
           <t>Cancel booking</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="inlineStr" s="0">
         <is>
           <t>verifyText</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="inlineStr" s="0">
         <is>
           <t>lblSuccessMessage</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" t="inlineStr" s="0">
         <is>
           <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="inlineStr" s="0">
         <is>
           <t>Verify success</t>
         </is>

</xml_diff>

<commit_message>
revert: remove excel template autofit update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -1,9 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <bookViews>
-    <workbookView activeTab="0"/>
-  </bookViews>
   <sheets>
     <sheet name="SCENARIOS" sheetId="1" r:id="rId1"/>
     <sheet name="Create New Booking" sheetId="2" r:id="rId2"/>
@@ -12,135 +9,86 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <sz val="11.0"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="darkGray"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-  </cellXfs>
-</styleSheet>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
-  <cols>
-    <col min="1" max="1" width="10.0" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="19.265625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="21.49609375" customWidth="true" bestFit="true"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="0">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="0">
+      <c r="B1" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="0">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ACTION</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="0">
+      <c r="D1" t="inlineStr">
         <is>
           <t>SCENARIOS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr" s="0">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="0">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Create New Booking</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="0">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Create booking room A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr" s="0">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="0">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Create New Booking</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="0">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Create booking room B</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr" s="0">
+      <c r="B4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="0">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Cancel Booking</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="0">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Cancel booking</t>
         </is>
@@ -152,271 +100,261 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G12"/>
-  <cols>
-    <col min="1" max="1" width="15.15625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="15.22265625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="18.078125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="34.265625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="12.01953125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="19.24609375" customWidth="true" bestFit="true"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="0">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Testcase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="0">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="0">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="0">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="0">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="0">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="0">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="0">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Login BRS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="0">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="0">
+      <c r="F2" t="inlineStr">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="0">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Login to BRS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="inlineStr" s="0">
+      <c r="C3" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="0">
+      <c r="D3" t="inlineStr">
         <is>
           <t>txtUsername</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="0">
+      <c r="E3" t="inlineStr">
         <is>
           <t>LOGIN_DATA[USERNAME]</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="0">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Input username</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="inlineStr" s="0">
+      <c r="C4" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="0">
+      <c r="D4" t="inlineStr">
         <is>
           <t>txtPassword</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="0">
+      <c r="E4" t="inlineStr">
         <is>
           <t>LOGIN_DATA[PASSWORD]</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="0">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Input password</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="0">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>btnLogin</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="0">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Click login</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="inlineStr" s="0">
+      <c r="C6" t="inlineStr">
         <is>
           <t>verifyDisplayed</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="0">
+      <c r="D6" t="inlineStr">
         <is>
           <t>lblDashboard</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="0">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Verify dashboard</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="0">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Create Booking</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="0">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr" s="0">
+      <c r="F7" t="inlineStr">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="0">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Create booking</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr" s="0">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>menuBooking</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr" s="0">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Open booking menu</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr" s="0">
+      <c r="C9" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="0">
+      <c r="D9" t="inlineStr">
         <is>
           <t>txtBookingTitle</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="0">
+      <c r="E9" t="inlineStr">
         <is>
           <t>BOOKING_DATA[BOOKING_TITLE]</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr" s="0">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Input title</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="0">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>btnRoomByName</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="0">
+      <c r="E10" t="inlineStr">
         <is>
           <t>BOOKING_DATA[ROOM_NAME]</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr" s="0">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Select room</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr" s="0">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>btnSubmitBooking</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr" s="0">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="inlineStr" s="0">
+      <c r="C12" t="inlineStr">
         <is>
           <t>verifyText</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="0">
+      <c r="D12" t="inlineStr">
         <is>
           <t>lblSuccessMessage</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="0">
+      <c r="E12" t="inlineStr">
         <is>
           <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr" s="0">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Verify success</t>
         </is>
@@ -428,215 +366,205 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G9"/>
-  <cols>
-    <col min="1" max="1" width="15.1484375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="10.0" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="18.078125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="34.265625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="12.01953125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="19.24609375" customWidth="true" bestFit="true"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="0">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Testcase</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="0">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="0">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="0">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="0">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="0">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="0">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="0">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Login BRS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="0">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="0">
+      <c r="F2" t="inlineStr">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="0">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Login to BRS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="inlineStr" s="0">
+      <c r="C3" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="0">
+      <c r="D3" t="inlineStr">
         <is>
           <t>txtUsername</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr" s="0">
+      <c r="E3" t="inlineStr">
         <is>
           <t>LOGIN_DATA[USERNAME]</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="0">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Input username</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="inlineStr" s="0">
+      <c r="C4" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="0">
+      <c r="D4" t="inlineStr">
         <is>
           <t>txtPassword</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="0">
+      <c r="E4" t="inlineStr">
         <is>
           <t>LOGIN_DATA[PASSWORD]</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="0">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Input password</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="0">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>btnLogin</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="0">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Click login</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="0">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Cancel Booking</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="0">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="0">
+      <c r="F6" t="inlineStr">
         <is>
           <t>BRS</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="0">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Cancel booking</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr" s="0">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>menuBooking</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="0">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Open booking menu</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr" s="0">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr" s="0">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>btnCancelBooking</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="0">
+      <c r="E8" t="inlineStr">
         <is>
           <t>BOOKING_DATA[BOOKING_ID]</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr" s="0">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Cancel booking</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr" s="0">
+      <c r="C9" t="inlineStr">
         <is>
           <t>verifyText</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="0">
+      <c r="D9" t="inlineStr">
         <is>
           <t>lblSuccessMessage</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="0">
+      <c r="E9" t="inlineStr">
         <is>
           <t>BOOKING_DATA[EXPECTED_MESSAGE]</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr" s="0">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Verify success</t>
         </is>

</xml_diff>

<commit_message>
feat: add object repository resolver
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Template Testing.xlsx
+++ b/src/test/resources/testdata/Template Testing.xlsx
@@ -11,12 +11,13 @@
     <sheet name="Cancel Booking" r:id="rId5" sheetId="3"/>
     <sheet name="LOGIN_DATA" r:id="rId6" sheetId="4"/>
     <sheet name="BOOKING_DATA" r:id="rId7" sheetId="5"/>
+    <sheet name="OBJECT_REPOSITORY" r:id="rId8" sheetId="6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="101">
   <si>
     <t>NO</t>
   </si>
@@ -241,6 +242,84 @@
   </si>
   <si>
     <t>BKG-002</t>
+  </si>
+  <si>
+    <t>XPath</t>
+  </si>
+  <si>
+    <t>//input[@id='username']</t>
+  </si>
+  <si>
+    <t>BRS username field</t>
+  </si>
+  <si>
+    <t>//input[@id='password']</t>
+  </si>
+  <si>
+    <t>BRS password field</t>
+  </si>
+  <si>
+    <t>//button[@id='login']</t>
+  </si>
+  <si>
+    <t>BRS login button</t>
+  </si>
+  <si>
+    <t>//h1[contains(text(),'Dashboard')]</t>
+  </si>
+  <si>
+    <t>Dashboard label</t>
+  </si>
+  <si>
+    <t>//span[text()='Booking']</t>
+  </si>
+  <si>
+    <t>Booking menu</t>
+  </si>
+  <si>
+    <t>//input[@name='bookingTitle']</t>
+  </si>
+  <si>
+    <t>Booking title input</t>
+  </si>
+  <si>
+    <t>//button[contains(text(),'{ROOM_NAME}')]</t>
+  </si>
+  <si>
+    <t>Dynamic room button</t>
+  </si>
+  <si>
+    <t>//button[@type='submit']</t>
+  </si>
+  <si>
+    <t>Submit booking button</t>
+  </si>
+  <si>
+    <t>//div[contains(@class,'success')]</t>
+  </si>
+  <si>
+    <t>Success message</t>
+  </si>
+  <si>
+    <t>//button[@data-booking='{BOOKING_ID}']</t>
+  </si>
+  <si>
+    <t>Dynamic cancel button</t>
+  </si>
+  <si>
+    <t>HRIS</t>
+  </si>
+  <si>
+    <t>//input[@id='employeeId']</t>
+  </si>
+  <si>
+    <t>HRIS username field</t>
+  </si>
+  <si>
+    <t>HRIS password field</t>
+  </si>
+  <si>
+    <t>HRIS login button</t>
   </si>
 </sst>
 </file>
@@ -954,4 +1033,210 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>